<commit_message>
Revise multi-department limitation text for clearer workshop explanation
Updated 6 cells across sheets 1 and 5 with simplified, elaborated limitation text:
- Changed from 'multi-department on 240 sites' to full explanation
- Now shows concrete examples (ADBI;BOD, CWRD;SARD, etc.)
- Clearly explains impact: departmental counts won't sum to bank-wide total
- Names path to resolution: RAC nominates primary department per site

Affected rows:
- S1 Bank-wide Oversight: rows 18, 20, 21, 33
- S5 Retention and Disposal: rows 20, 27

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AV4qAXX91hebiyNkkAdbcm
</commit_message>
<xml_diff>
--- a/EDRMS_Utilization_Dashboard_Gap_Checker_2026-08-26.xlsx
+++ b/EDRMS_Utilization_Dashboard_Gap_Checker_2026-08-26.xlsx
@@ -1308,7 +1308,9 @@
       <c r="F18" s="2" t="n"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>• Can use CG Workspace report &gt; filter EDRMS Site Type = 'EDRMS Project Site' &gt; group by Department &gt; count rows. Same multi-department limitation as the Department column.</t>
+          <t>• Can use CG Workspace report &gt; filter EDRMS Site Type = 'EDRMS Project Site' &gt; group by Department &gt; count rows.
+Limitation: Some sites in the workspace report carry multiple departments, semicolon separated (ADBI;BOD, CWRD;SARD, ADBI;BOD;CSD;CWRD;SARD). Departmental counts will not sum to the bank-wide total until RAC nominates one primary department per site.
+Needs: RAC production export</t>
         </is>
       </c>
       <c r="H18" s="19" t="n"/>
@@ -1379,7 +1381,8 @@
       <c r="G20" s="2" t="inlineStr">
         <is>
           <t>• Existing in the database. public."Records" &gt; join SiteUrl to the CG export &gt; group by Department &gt; count distinct (ListId, ItemId).
-• Limitation: the department comes from CG, so this inherits the multi-department problem on 240 sites.</t>
+Limitation: Some sites in the workspace report carry multiple departments, semicolon separated (ADBI;BOD, CWRD;SARD, ADBI;BOD;CSD;CWRD;SARD). Departmental counts will not sum to the bank-wide total until RAC nominates one primary department per site.
+Needs: RAC production export</t>
         </is>
       </c>
       <c r="H20" s="19" t="n"/>
@@ -1415,7 +1418,9 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>• Existing in the database. HasPhysical grouped by Department through the same SiteUrl join. Same multi-department limitation.</t>
+          <t>• Existing in the database. HasPhysical grouped by Department through the same SiteUrl join.
+Limitation: Some sites in the workspace report carry multiple departments, semicolon separated (ADBI;BOD, CWRD;SARD, ADBI;BOD;CSD;CWRD;SARD). Departmental counts will not sum to the bank-wide total until RAC nominates one primary department per site.
+Needs: RAC production export</t>
         </is>
       </c>
       <c r="H21" s="19" t="n"/>
@@ -1778,7 +1783,9 @@
       <c r="F33" s="2" t="n"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>• Can use CG Workspace report &gt; distinct Department over the compliant sites. Same multi-department limitation as the Department column.</t>
+          <t>• Can use CG Workspace report &gt; distinct Department over the compliant sites.
+Limitation: Some sites in the workspace report carry multiple departments, semicolon separated (ADBI;BOD, CWRD;SARD, ADBI;BOD;CSD;CWRD;SARD). Departmental counts will not sum to the bank-wide total until RAC nominates one primary department per site.
+Needs: RAC production export</t>
         </is>
       </c>
       <c r="H33" s="31" t="e">
@@ -3319,18 +3326,6 @@
       </c>
       <c r="H80" s="19" t="n"/>
     </row>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
     <row r="93">
       <c r="E93" s="45" t="n"/>
     </row>
@@ -23914,7 +23909,9 @@
       <c r="F20" s="2" t="n"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>• Can use CG Workspace report &gt; Department through the SiteUrl join. Same multi-department limitation.</t>
+          <t>• Can use CG Workspace report &gt; Department through the SiteUrl join.
+Limitation: Some sites in the workspace report carry multiple departments, semicolon separated (ADBI;BOD, CWRD;SARD, ADBI;BOD;CSD;CWRD;SARD). Departmental counts will not sum to the bank-wide total until RAC nominates one primary department per site.
+Needs: RAC production export</t>
         </is>
       </c>
       <c r="H20" s="2" t="n"/>
@@ -24150,7 +24147,9 @@
       <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>• Can use CG Workspace report &gt; Department through the SiteUrl join. Same multi-department limitation.</t>
+          <t>• Can use CG Workspace report &gt; Department through the SiteUrl join.
+Limitation: Some sites in the workspace report carry multiple departments, semicolon separated (ADBI;BOD, CWRD;SARD, ADBI;BOD;CSD;CWRD;SARD). Departmental counts will not sum to the bank-wide total until RAC nominates one primary department per site.
+Needs: RAC production export</t>
         </is>
       </c>
       <c r="H27" s="2" t="n"/>

</xml_diff>